<commit_message>
Ground the eval judges in retrieved passages; respond examples; tracing fixes
- Evals: correctness now judges the reply against the passages the agent
  was shown (read from the checkpoint history) and the conversation;
  statements about the assistant, the ticket and urgency are not checked.
  completeness judges against the expected answer. Greeting turns are
  not judged.
- Datasets: drop instruction text used as reference context, drop
  order-dependent follow-up turns, replace openers the knowledge base
  answers, add recall-first-question-ar and the happy_path suite.
- Respond: few-shot examples per step, including a wrong-passage case
  and a partial-coverage case.
- Router: conversation meta-questions go to ask; chat wording instead of
  email wording in the searching rules.
- Tracing: keep only traces that carry a session id, name the LLM spans
  by node and record reasoning on a span per attempt.
</commit_message>
<xml_diff>
--- a/sheets/attachments.xlsx
+++ b/sheets/attachments.xlsx
@@ -1,23 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="15324" windowHeight="6948" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="attachments" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="attachments" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,7 +25,17 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,15 +55,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -417,13 +429,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="1" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -448,7 +457,76 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>T-MOCK-20261020103942-0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>debug.log</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>http://localhost:8000/chat/attachments/VGUI-Z74RweNbr0pRty1PuQzQUZoPGdp</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-10-20T07:36:21+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>T-MOCK-20261020115633-0001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>debug.log</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>http://localhost:8000/chat/attachments/0iepHJ5YEzWkqzJKYimGh5TJxO6QiuBW</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-10-20T08:56:07+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>T-MOCK-20261020151240-0001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>23828.jpg</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>http://localhost:8000/chat/attachments/RtJl1x-FFUaz3RDEpLB4qFkRs8KeIfWd</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-10-20T12:03:14+00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>